<commit_message>
Change wording 'amount' and 'capacity' to 'nominal_capacity'
</commit_message>
<xml_diff>
--- a/tests/files/input_data.xlsx
+++ b/tests/files/input_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Projekte\3-152-24-HBl_PyFlex\2 Inhalte\10 Arbeitspaket 5\pyromof-non-tabular\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Projekte\3-152-24-HBl_PyFlex\2 Inhalte\10 Arbeitspaket 5\pyromof-non-tabular\tests\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACA793D-7D79-4119-8EC0-4431E17C54CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9D6AB1-C2E4-4BDC-9E1F-4569B39519FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{46330B2F-E85C-4459-B76B-09B0963C0FC2}"/>
+    <workbookView xWindow="3555" yWindow="-19170" windowWidth="23250" windowHeight="13890" activeTab="3" xr2:uid="{46330B2F-E85C-4459-B76B-09B0963C0FC2}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="8" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="63">
   <si>
     <t>biomass</t>
   </si>
@@ -64,9 +64,6 @@
     <t>profile</t>
   </si>
   <si>
-    <t>capacity</t>
-  </si>
-  <si>
     <t>invest</t>
   </si>
   <si>
@@ -118,9 +115,6 @@
     <t>co2_market</t>
   </si>
   <si>
-    <t>amount</t>
-  </si>
-  <si>
     <t>profile_heat</t>
   </si>
   <si>
@@ -242,6 +236,9 @@
   </si>
   <si>
     <t>minimum</t>
+  </si>
+  <si>
+    <t>nominal_capacity</t>
   </si>
 </sst>
 </file>
@@ -720,15 +717,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2">
         <v>0.05</v>
@@ -752,65 +749,65 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" s="20">
         <v>-1000</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="11">
         <v>1000</v>
@@ -822,27 +819,27 @@
         <v>-125</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F4" s="11">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -865,7 +862,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -874,31 +871,31 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
@@ -909,60 +906,60 @@
         <v>2</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2" s="11">
         <v>1000000000000000</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="20">
         <v>250</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D3" s="22">
         <v>100000000000</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H3" s="20">
         <v>10000000</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -993,99 +990,99 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="O1" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="P1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="M1" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>59</v>
-      </c>
       <c r="Q1" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="R1" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="U1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="V1" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="S1" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="T1" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="U1" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="V1" s="12" t="s">
-        <v>53</v>
-      </c>
       <c r="W1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="X1" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="Y1" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
         <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>19</v>
       </c>
       <c r="G2" s="3">
         <v>1000</v>
@@ -1136,30 +1133,30 @@
         <v>0</v>
       </c>
       <c r="X2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Y2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:25" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>19</v>
       </c>
       <c r="G3" s="15">
         <v>1000</v>
@@ -1210,10 +1207,10 @@
         <v>1000</v>
       </c>
       <c r="X3" s="11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Y3" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
@@ -1245,43 +1242,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1301,13 +1298,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>